<commit_message>
Plan Taquería F2: revisión adversarial (0 B · 5 M · 10 m; mayores arreglados, cifras sin mover) + mismos arreglos en la FAQ de la landing
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-taqueria/checklist-apertura-taqueria.xlsx
+++ b/astro-site/public/dl/plan-negocio-taqueria/checklist-apertura-taqueria.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>El plan compra la tortilla. Hacerla en casa pide molino, cocedor y tortilladora, sitio en la cocina y un tortillero: por coste sólo compensa por encima de unas 700 tortillas al día (la calculadora del pack hace la cuenta con tus precios). Si la haces tú, el local tiene que caberla</t>
+          <t>El plan compra la tortilla. Hacerla en casa pide molino, cocedor y tortilladora, sitio en la cocina y un tortillero: por coste sólo compensa por encima de unas 700 tortillas al día (la calculadora del pack hace la cuenta con tus precios). Si la haces tú, el molino y la tortilladora tienen que caber en el local</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Los recipientes de plástico de un solo uso para llevar se cobran aparte en el tique (Ley 7/2022, art. 55). Las bandejas de cartón no son plástico; las de aluminio, pregúntalo a tu proveedor</t>
+          <t>Los recipientes de plástico de un solo uso para llevar se cobran aparte en el tique (Ley 7/2022, art. 55). Las bandejas de cartón sin recubrimiento de plástico no lo son; las de aluminio, pregúntalo a tu proveedor</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Tortilla de maíz nixtamalizado con lote y fecha, recibida a la temperatura que marque su etiqueta y anotada. Pide muestra a dos fabricantes y precio por caja: el plan la estima, no la ha leído en una tarifa</t>
+          <t>Tortilla de maíz nixtamalizado con lote y fecha, recibida a la temperatura que marque su etiqueta y anotada. Pide muestra a dos fabricantes y precio por caja: el plan la estima con un precio de referencia: pon el tuyo</t>
         </is>
       </c>
     </row>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Septiembre, noviembre y diciembre son los picos del año: prepara el cuadrante y el stock con tiempo</t>
+          <t>Diciembre es el pico del año y septiembre y noviembre traen las fechas mexicanas: prepara el cuadrante y el stock con tiempo</t>
         </is>
       </c>
     </row>

</xml_diff>